<commit_message>
Add stock analysis Excel
</commit_message>
<xml_diff>
--- a/daily/20260309/20260309_小斐选股_行业 top20.xlsx
+++ b/daily/20260309/20260309_小斐选股_行业 top20.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Z1160"/>
+  <dimension ref="A1:Z1163"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="6.83203125" customWidth="1"/>
@@ -84746,9 +84746,249 @@
         <v>否</v>
       </c>
     </row>
+    <row r="1161">
+      <c r="A1161" t="str">
+        <v>小金属</v>
+      </c>
+      <c r="B1161" t="str">
+        <v>持仓</v>
+      </c>
+      <c r="C1161" t="str">
+        <v>600392.SH</v>
+      </c>
+      <c r="D1161" t="str">
+        <v>盛和资源</v>
+      </c>
+      <c r="E1161" t="str">
+        <v>588</v>
+      </c>
+      <c r="F1161" t="str">
+        <v>156.84</v>
+      </c>
+      <c r="G1161" t="str">
+        <v>2.21</v>
+      </c>
+      <c r="H1161" t="str">
+        <v>27.52</v>
+      </c>
+      <c r="I1161" t="str">
+        <v>-1.18</v>
+      </c>
+      <c r="J1161" t="str">
+        <v>28.10</v>
+      </c>
+      <c r="K1161" t="str">
+        <v>29.84</v>
+      </c>
+      <c r="L1161" t="str">
+        <v>-5.83</v>
+      </c>
+      <c r="M1161" t="str">
+        <v>0.0</v>
+      </c>
+      <c r="N1161" t="str">
+        <v>0.95</v>
+      </c>
+      <c r="O1161" t="str">
+        <v>✗</v>
+      </c>
+      <c r="P1161" t="str">
+        <v>✗</v>
+      </c>
+      <c r="Q1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="R1161" t="str">
+        <v>✗</v>
+      </c>
+      <c r="S1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="T1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="U1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="V1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="W1161" t="str">
+        <v>✗</v>
+      </c>
+      <c r="X1161" t="str">
+        <v>✓</v>
+      </c>
+      <c r="Y1161">
+        <v>6</v>
+      </c>
+      <c r="Z1161" t="str">
+        <v>否</v>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="str">
+        <v>小金属</v>
+      </c>
+      <c r="B1162" t="str">
+        <v>持仓</v>
+      </c>
+      <c r="C1162" t="str">
+        <v>000969.SZ</v>
+      </c>
+      <c r="D1162" t="str">
+        <v>安泰科技</v>
+      </c>
+      <c r="E1162" t="str">
+        <v>268</v>
+      </c>
+      <c r="F1162" t="str">
+        <v>29.22</v>
+      </c>
+      <c r="G1162" t="str">
+        <v>2.42</v>
+      </c>
+      <c r="H1162" t="str">
+        <v>23.75</v>
+      </c>
+      <c r="I1162" t="str">
+        <v>-1.62</v>
+      </c>
+      <c r="J1162" t="str">
+        <v>24.07</v>
+      </c>
+      <c r="K1162" t="str">
+        <v>24.64</v>
+      </c>
+      <c r="L1162" t="str">
+        <v>-2.31</v>
+      </c>
+      <c r="M1162" t="str">
+        <v>33.9</v>
+      </c>
+      <c r="N1162" t="str">
+        <v>0.96</v>
+      </c>
+      <c r="O1162" t="str">
+        <v>✗</v>
+      </c>
+      <c r="P1162" t="str">
+        <v>✗</v>
+      </c>
+      <c r="Q1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="R1162" t="str">
+        <v>✗</v>
+      </c>
+      <c r="S1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="T1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="U1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="V1162" t="str">
+        <v>✗</v>
+      </c>
+      <c r="W1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="X1162" t="str">
+        <v>✓</v>
+      </c>
+      <c r="Y1162">
+        <v>6</v>
+      </c>
+      <c r="Z1162" t="str">
+        <v>否</v>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="str">
+        <v>电气设备</v>
+      </c>
+      <c r="B1163" t="str">
+        <v>持仓</v>
+      </c>
+      <c r="C1163" t="str">
+        <v>002270.SZ</v>
+      </c>
+      <c r="D1163" t="str">
+        <v>华明装备</v>
+      </c>
+      <c r="E1163" t="str">
+        <v>301</v>
+      </c>
+      <c r="F1163" t="str">
+        <v>21.93</v>
+      </c>
+      <c r="G1163" t="str">
+        <v>4.67</v>
+      </c>
+      <c r="H1163" t="str">
+        <v>36.65</v>
+      </c>
+      <c r="I1163" t="str">
+        <v>-0.65</v>
+      </c>
+      <c r="J1163" t="str">
+        <v>35.68</v>
+      </c>
+      <c r="K1163" t="str">
+        <v>35.08</v>
+      </c>
+      <c r="L1163" t="str">
+        <v>1.71</v>
+      </c>
+      <c r="M1163" t="str">
+        <v>70.5</v>
+      </c>
+      <c r="N1163" t="str">
+        <v>0.86</v>
+      </c>
+      <c r="O1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="P1163" t="str">
+        <v>✗</v>
+      </c>
+      <c r="Q1163" t="str">
+        <v>✗</v>
+      </c>
+      <c r="R1163" t="str">
+        <v>✗</v>
+      </c>
+      <c r="S1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="T1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="U1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="V1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="W1163" t="str">
+        <v>✗</v>
+      </c>
+      <c r="X1163" t="str">
+        <v>✓</v>
+      </c>
+      <c r="Y1163">
+        <v>6</v>
+      </c>
+      <c r="Z1163" t="str">
+        <v>是</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Z1160"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Z1163"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>